<commit_message>
Apply Omni Convert Patches 36, 36.5, and 37
</commit_message>
<xml_diff>
--- a/smoke_test_output_example/pdf_to_xlsx/sample.xlsx
+++ b/smoke_test_output_example/pdf_to_xlsx/sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -459,174 +459,6 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>